<commit_message>
2026 02 26 kinda realise
</commit_message>
<xml_diff>
--- a/borchestra_chars.xlsx
+++ b/borchestra_chars.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B13"/>
+  <dimension ref="A1:B14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -431,144 +431,156 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Coral_CH</t>
+          <t>AtlasGF_CH</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Coral</t>
+          <t>Atlas</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Drubberslunger_CH</t>
+          <t>BiersalGF_CH</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Drubberslunger</t>
+          <t>Biersal</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Flodhest_CH</t>
+          <t>DahliaGF_CH</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Flodhest</t>
+          <t>Dahlia</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Ham_CH</t>
+          <t>GreasyDerekGF_CH</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Ham</t>
+          <t>Derek</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Knotty_CH</t>
+          <t>FelGF_CH</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Knotty</t>
+          <t>Fel</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Pavel&amp;Perseus_CH</t>
+          <t>GourdGF_CH</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Pavel&amp;Perseus</t>
+          <t>Gourd</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Reyes_CH</t>
+          <t>OathsGF_CH</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Reyes</t>
+          <t>Oaths</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Serpent_CH</t>
+          <t>OMEGARAGERGF_CH</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Serpent</t>
+          <t>OMEGARAGER</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Sulfuric_CH</t>
+          <t>GreasyQuarellGF_CH</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Sulfuric</t>
+          <t>Quarell</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Vertus_CH</t>
+          <t>Red_RagerGF_CH</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Vertus</t>
+          <t>RedRager</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>WormWoomb_CH</t>
+          <t>StainGF_CH</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>WormWomb</t>
+          <t>Stain</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>BirthedWomb_CH</t>
+          <t>SwellGF_CH</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>BirthedWomb</t>
+          <t>Swell</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>WhaleGF_CH</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>Whale</t>
         </is>
       </c>
     </row>

</xml_diff>